<commit_message>
Master database: PTIN confirmed; REDF and JC Flowers as funders and partners
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rb4ZTXZXZvRymPmEXq9dPj
</commit_message>
<xml_diff>
--- a/jobsearch/career_database.xlsx
+++ b/jobsearch/career_database.xlsx
@@ -2739,7 +2739,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>City of New York; REDF; JC Flowers; agencies; employers</t>
+          <t>City of New York; REDF and JC Flowers (funders and partners); agencies; employers</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Compile Form 990 returns for multiple nonprofits and prepare and file business and individual tax returns, including dozens of state and local filings; IRS-registered tax preparer (confirm PTIN).</t>
+          <t>Compile Form 990 returns for multiple nonprofits and prepare and file business and individual tax returns, including dozens of state and local filings; IRS-registered tax preparer with an active PTIN.</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Former FINRA Series 7 &amp; 63; former Life, Accident &amp; Health licenses; IRS-registered tax preparer (confirm PTIN)</t>
+          <t>IRS-registered tax preparer (active PTIN); former FINRA Series 7 &amp; 63; former Life, Accident &amp; Health licenses</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">

</xml_diff>

<commit_message>
EngageWell: concrete fundraising bullets, harm-reduction framing in letter; master list fundraising evidence
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rb4ZTXZXZvRymPmEXq9dPj
</commit_message>
<xml_diff>
--- a/jobsearch/career_database.xlsx
+++ b/jobsearch/career_database.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5221,6 +5221,120 @@
       <c r="K83" s="2" t="inlineStr">
         <is>
           <t>Stated by Clavel, Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>E083</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Fundraising</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Prospect Development &amp; Solicitation</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Identified and prioritized prospects, developed proposals, and personally led solicitation of the highest-value donors, foundations, and corporate partners (REDF, JC Flowers).</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>$400K+ raised (FY23–)</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Osborne Association</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>VP Business Development &amp; Social Ventures</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Nonprofit</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>prospect research; proposals; solicitation; major donors; REDF; JC Flowers</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Original Advancement resume (Clavel)</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>Stated by Clavel</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>E084</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Fundraising</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Board-Led Cultivation &amp; Stewardship</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Partnered with the CEO, Board, and Fund Development Committee on donor cultivation and stewardship; deployed board members in cultivation; co-led annual fundraising events that exceeded revenue targets.</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Annual events</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Osborne Association</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>VP Business Development &amp; Social Ventures</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Nonprofit</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>cultivation; stewardship; board engagement; fundraising events; Fund Development Committee</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Original Advancement resume (Clavel)</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>Stated by Clavel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
EngageWell: remove fundraising figures; record no-fundraising-numbers preference in master list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rb4ZTXZXZvRymPmEXq9dPj
</commit_message>
<xml_diff>
--- a/jobsearch/career_database.xlsx
+++ b/jobsearch/career_database.xlsx
@@ -7562,7 +7562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7764,6 +7764,23 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Fundraising figures</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Do not state fundraising dollar amounts on resumes or letters (Clavel, 2026-10-30). Describe fundraising qualitatively; contract values (e.g., $10M+ contracts) are separate.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Clavel has also cited $400K+ (FY23–) and $40M+ over 10 years; keep off documents unless asked</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Master list: HR evidence (workforce program HR, HR manuals, NY employment law)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rb4ZTXZXZvRymPmEXq9dPj
</commit_message>
<xml_diff>
--- a/jobsearch/career_database.xlsx
+++ b/jobsearch/career_database.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5335,6 +5335,177 @@
       <c r="K85" s="2" t="inlineStr">
         <is>
           <t>Stated by Clavel</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>E085</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Workforce Program HR Oversight</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Ran HR for a workforce program with oversight of hundreds of workers: hiring, supervision, and handling of employee complaints.</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Hundreds of workers</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Osborne Association</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>VP Business Development &amp; Social Ventures</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Workforce / human services</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>HR; hiring; supervision; employee relations; complaints; workforce program</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Clavel (chat, Oct 2026)</t>
+        </is>
+      </c>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>Stated by Clavel, Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>E086</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>HR Policy &amp; Manuals</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>Created HR manuals for the department and for Osborne.</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>Department and organization-wide</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Osborne Association</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>VP Business Development &amp; Social Ventures</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Nonprofit</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>HR manuals; policies; employee handbook</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Clavel (chat, Oct 2026)</t>
+        </is>
+      </c>
+      <c r="K87" s="2" t="inlineStr">
+        <is>
+          <t>Stated by Clavel, Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>E087</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>HR / Compliance</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>NY Employment Law</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Applied New York employment law in managing hiring, supervision, compensation, and employee complaints.</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Osborne Association</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>VP Business Development &amp; Social Ventures</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Nonprofit</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>NY employment law; compliance; employee relations</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Clavel (chat, Oct 2026)</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>Stated by Clavel, Oct 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master list: landlord relationships, retirement plans, safety plans; flag franchise-count conflict
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rb4ZTXZXZvRymPmEXq9dPj
</commit_message>
<xml_diff>
--- a/jobsearch/career_database.xlsx
+++ b/jobsearch/career_database.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K88"/>
+  <dimension ref="A1:K91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5504,6 +5504,177 @@
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>Stated by Clavel, Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>E088</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Facilities</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Landlord &amp; Lease Relationships</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Managed landlord relationships, facilities, insurance, utilities, and vendor contracts across multiple locations.</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Multi-location</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Fitness Collective</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder / CEO</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Fitness / franchise</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>landlord; leases; facilities; utilities; vendors</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Clavel (chat, Oct 2026)</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>Stated by Clavel, Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>E089</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Benefits</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Retirement Plan Design &amp; Administration</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Created and administered retirement plans, including at Alluel Logistics and for Maroon Strategist clients.</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Multiple organizations</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Alluel Logistics / Maroon Strategist</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>VP Operations / Fractional CFO</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Cross-industry</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>retirement plans; 401(k); benefits administration</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Clavel (chat, Oct 2026)</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>Stated by Clavel, Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>E090</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Safety &amp; Risk</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Safety Plans</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Wrote safety plans and procedures for Fitness Collective and its five franchise locations.</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Company + 5 franchises</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Fitness Collective</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Co-Founder / CEO</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Fitness / franchise</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>safety plans; emergency preparedness; risk management; franchise operations</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Clavel (chat, Oct 2026)</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
         <is>
           <t>Stated by Clavel, Oct 2026</t>
         </is>
@@ -6944,7 +7115,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Clavel uses three additional locations (current resumes)</t>
+          <t>Open: Clavel cited "three additional locations" (resumes) and "5 franchises we ran" (chat, 2026-10-30); confirm which to use</t>
         </is>
       </c>
     </row>

</xml_diff>